<commit_message>
Verify GitHub CI results and finalize original-form submission report
</commit_message>
<xml_diff>
--- a/docs/Report5_UnitTest.xlsx
+++ b/docs/Report5_UnitTest.xlsx
@@ -7787,7 +7787,7 @@
     <row r="14" spans="1:23" ht="13.5" customHeight="1">
       <c r="A14" s="221"/>
       <c r="B14" s="93" t="str">
-        <v>Input / state</v>
+        <v>Input/state : HTTP</v>
       </c>
       <c r="C14" s="94"/>
       <c r="D14" s="95"/>
@@ -7813,7 +7813,7 @@
       <c r="B15" s="93"/>
       <c r="C15" s="94"/>
       <c r="D15" s="95" t="str">
-        <v>fullName=""</v>
+        <v>name="":3</v>
       </c>
       <c r="E15" s="100"/>
       <c r="F15" s="186" t="str">
@@ -7842,7 +7842,7 @@
       <c r="B16" s="93"/>
       <c r="C16" s="94"/>
       <c r="D16" s="95" t="str">
-        <v>email=""</v>
+        <v>email="":3</v>
       </c>
       <c r="E16" s="100"/>
       <c r="F16" s="186"/>
@@ -7871,7 +7871,7 @@
       <c r="B17" s="93"/>
       <c r="C17" s="94"/>
       <c r="D17" s="95" t="str">
-        <v>password=""</v>
+        <v>pwd="":3</v>
       </c>
       <c r="E17" s="100"/>
       <c r="F17" s="186"/>
@@ -7900,7 +7900,7 @@
       <c r="B18" s="93"/>
       <c r="C18" s="94"/>
       <c r="D18" s="95" t="str">
-        <v>role=""</v>
+        <v>role="":3</v>
       </c>
       <c r="E18" s="100"/>
       <c r="F18" s="186"/>
@@ -7929,7 +7929,7 @@
       <c r="B19" s="93"/>
       <c r="C19" s="94"/>
       <c r="D19" s="342" t="str">
-        <v>role=ADMIN</v>
+        <v>role=ADMIN:3</v>
       </c>
       <c r="E19" s="342"/>
       <c r="F19" s="186"/>
@@ -7958,7 +7958,7 @@
       <c r="B20" s="93"/>
       <c r="C20" s="94"/>
       <c r="D20" s="95" t="str">
-        <v>password=Aa1234!</v>
+        <v>pwd=Aa1234!:3</v>
       </c>
       <c r="E20" s="100"/>
       <c r="F20" s="186"/>
@@ -7987,7 +7987,7 @@
       <c r="B21" s="93"/>
       <c r="C21" s="94"/>
       <c r="D21" s="95" t="str">
-        <v>password=aa12345!</v>
+        <v>pwd=aa12345!:3</v>
       </c>
       <c r="E21" s="100"/>
       <c r="F21" s="186"/>
@@ -8016,7 +8016,7 @@
       <c r="B22" s="93"/>
       <c r="C22" s="94"/>
       <c r="D22" s="95" t="str">
-        <v>password=AA12345!</v>
+        <v>pwd=AA12345!:3</v>
       </c>
       <c r="E22" s="100"/>
       <c r="F22" s="186"/>
@@ -8045,7 +8045,7 @@
       <c r="B23" s="93"/>
       <c r="C23" s="94"/>
       <c r="D23" s="95" t="str">
-        <v>no digit/special</v>
+        <v>no digit/special:3</v>
       </c>
       <c r="E23" s="100"/>
       <c r="F23" s="186"/>
@@ -8074,7 +8074,7 @@
       <c r="B24" s="93"/>
       <c r="C24" s="94"/>
       <c r="D24" s="95" t="str">
-        <v>SQL query rejects</v>
+        <v>SQL error:7</v>
       </c>
       <c r="E24" s="100"/>
       <c r="F24" s="186"/>
@@ -8103,7 +8103,7 @@
       <c r="B25" s="93"/>
       <c r="C25" s="94"/>
       <c r="D25" s="95" t="str">
-        <v>email exists</v>
+        <v>email exists:3</v>
       </c>
       <c r="E25" s="100"/>
       <c r="F25" s="186"/>
@@ -8132,7 +8132,7 @@
       <c r="B26" s="93"/>
       <c r="C26" s="94"/>
       <c r="D26" s="95" t="str">
-        <v>phone=123</v>
+        <v>phone=123:3</v>
       </c>
       <c r="E26" s="100"/>
       <c r="F26" s="186"/>
@@ -8161,7 +8161,7 @@
       <c r="B27" s="93"/>
       <c r="C27" s="94"/>
       <c r="D27" s="95" t="str">
-        <v>phone exists</v>
+        <v>phone exists:3</v>
       </c>
       <c r="E27" s="100"/>
       <c r="F27" s="186"/>
@@ -8190,7 +8190,7 @@
       <c r="B28" s="93"/>
       <c r="C28" s="94"/>
       <c r="D28" s="95" t="str">
-        <v>role=freelancer</v>
+        <v>role=free:2</v>
       </c>
       <c r="E28" s="100"/>
       <c r="F28" s="186"/>
@@ -8219,7 +8219,7 @@
       <c r="B29" s="93"/>
       <c r="C29" s="94"/>
       <c r="D29" s="95" t="str">
-        <v>role=EMPLOYER</v>
+        <v>role=EMP:2</v>
       </c>
       <c r="E29" s="100"/>
       <c r="F29" s="186"/>
@@ -8299,53 +8299,53 @@
       <c r="B32" s="112"/>
       <c r="C32" s="113"/>
       <c r="D32" s="114" t="str">
-        <v>HTTP code (C5)</v>
+        <v>HTTP as input</v>
       </c>
       <c r="E32" s="115"/>
-      <c r="F32" s="186" t="n">
-        <v>3</v>
-      </c>
-      <c r="G32" s="186" t="n">
-        <v>3</v>
-      </c>
-      <c r="H32" s="186" t="n">
-        <v>3</v>
-      </c>
-      <c r="I32" s="186" t="n">
-        <v>3</v>
-      </c>
-      <c r="J32" s="186" t="n">
-        <v>3</v>
-      </c>
-      <c r="K32" s="186" t="n">
-        <v>3</v>
-      </c>
-      <c r="L32" s="186" t="n">
-        <v>3</v>
-      </c>
-      <c r="M32" s="186" t="n">
-        <v>3</v>
-      </c>
-      <c r="N32" s="186" t="n">
-        <v>3</v>
-      </c>
-      <c r="O32" s="186" t="n">
-        <v>7</v>
-      </c>
-      <c r="P32" s="186" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q32" s="186" t="n">
-        <v>3</v>
-      </c>
-      <c r="R32" s="186" t="n">
-        <v>3</v>
-      </c>
-      <c r="S32" s="186" t="n">
-        <v>2</v>
-      </c>
-      <c r="T32" s="220" t="n">
-        <v>2</v>
+      <c r="F32" s="186" t="str">
+        <v>O</v>
+      </c>
+      <c r="G32" s="186" t="str">
+        <v>O</v>
+      </c>
+      <c r="H32" s="186" t="str">
+        <v>O</v>
+      </c>
+      <c r="I32" s="186" t="str">
+        <v>O</v>
+      </c>
+      <c r="J32" s="186" t="str">
+        <v>O</v>
+      </c>
+      <c r="K32" s="186" t="str">
+        <v>O</v>
+      </c>
+      <c r="L32" s="186" t="str">
+        <v>O</v>
+      </c>
+      <c r="M32" s="186" t="str">
+        <v>O</v>
+      </c>
+      <c r="N32" s="186" t="str">
+        <v>O</v>
+      </c>
+      <c r="O32" s="186" t="str">
+        <v>O</v>
+      </c>
+      <c r="P32" s="186" t="str">
+        <v>O</v>
+      </c>
+      <c r="Q32" s="186" t="str">
+        <v>O</v>
+      </c>
+      <c r="R32" s="186" t="str">
+        <v>O</v>
+      </c>
+      <c r="S32" s="186" t="str">
+        <v>O</v>
+      </c>
+      <c r="T32" s="220" t="str">
+        <v>O</v>
       </c>
       <c r="U32"/>
       <c r="V32"/>
@@ -9202,7 +9202,7 @@
     <row r="14" spans="1:23" ht="13.5" customHeight="1">
       <c r="A14" s="221"/>
       <c r="B14" s="93" t="str">
-        <v>Input / state</v>
+        <v>Input/state : HTTP</v>
       </c>
       <c r="C14" s="94"/>
       <c r="D14" s="95"/>
@@ -9228,7 +9228,7 @@
       <c r="B15" s="93"/>
       <c r="C15" s="94"/>
       <c r="D15" s="95" t="str">
-        <v>email=""</v>
+        <v>email="":3</v>
       </c>
       <c r="E15" s="100"/>
       <c r="F15" s="97" t="str">
@@ -9257,7 +9257,7 @@
       <c r="B16" s="93"/>
       <c r="C16" s="94"/>
       <c r="D16" s="95" t="str">
-        <v>code=""</v>
+        <v>code="":3</v>
       </c>
       <c r="E16" s="100"/>
       <c r="F16" s="97"/>
@@ -9286,7 +9286,7 @@
       <c r="B17" s="93"/>
       <c r="C17" s="94"/>
       <c r="D17" s="95" t="str">
-        <v>user not found</v>
+        <v>user not found:6</v>
       </c>
       <c r="E17" s="100"/>
       <c r="F17" s="97"/>
@@ -9315,7 +9315,7 @@
       <c r="B18" s="93"/>
       <c r="C18" s="94"/>
       <c r="D18" s="95" t="str">
-        <v>verified=true</v>
+        <v>verified=true:1</v>
       </c>
       <c r="E18" s="100"/>
       <c r="F18" s="97"/>
@@ -9344,7 +9344,7 @@
       <c r="B19" s="93"/>
       <c r="C19" s="94"/>
       <c r="D19" s="342" t="str">
-        <v>code=wrong</v>
+        <v>code=wrong:3</v>
       </c>
       <c r="E19" s="342"/>
       <c r="F19" s="97"/>
@@ -9373,7 +9373,7 @@
       <c r="B20" s="93"/>
       <c r="C20" s="94"/>
       <c r="D20" s="95" t="str">
-        <v>code=used</v>
+        <v>code=used:3</v>
       </c>
       <c r="E20" s="100"/>
       <c r="F20" s="97"/>
@@ -9402,7 +9402,7 @@
       <c r="B21" s="93"/>
       <c r="C21" s="94"/>
       <c r="D21" s="95" t="str">
-        <v>expiry=now-1ms</v>
+        <v>expiry=now-1ms:3</v>
       </c>
       <c r="E21" s="100"/>
       <c r="F21" s="97"/>
@@ -9431,7 +9431,7 @@
       <c r="B22" s="93"/>
       <c r="C22" s="94"/>
       <c r="D22" s="95" t="str">
-        <v>expiry=now</v>
+        <v>expiry=now:1</v>
       </c>
       <c r="E22" s="100"/>
       <c r="F22" s="97"/>
@@ -9460,7 +9460,7 @@
       <c r="B23" s="93"/>
       <c r="C23" s="94"/>
       <c r="D23" s="95" t="str">
-        <v>expiry=now+1ms</v>
+        <v>expiry=now+1ms:1</v>
       </c>
       <c r="E23" s="100"/>
       <c r="F23" s="97"/>
@@ -9489,7 +9489,7 @@
       <c r="B24" s="93"/>
       <c r="C24" s="94"/>
       <c r="D24" s="95" t="str">
-        <v>expiry=now+10m</v>
+        <v>expiry=now+10m:1</v>
       </c>
       <c r="E24" s="100"/>
       <c r="F24" s="97"/>
@@ -9518,7 +9518,7 @@
       <c r="B25" s="93"/>
       <c r="C25" s="94"/>
       <c r="D25" s="95" t="str">
-        <v>query1 rejects</v>
+        <v>query1 error:7</v>
       </c>
       <c r="E25" s="100"/>
       <c r="F25" s="97"/>
@@ -9547,7 +9547,7 @@
       <c r="B26" s="93"/>
       <c r="C26" s="94"/>
       <c r="D26" s="95" t="str">
-        <v>query2 rejects</v>
+        <v>query2 error:7</v>
       </c>
       <c r="E26" s="100"/>
       <c r="F26" s="97"/>
@@ -9576,7 +9576,7 @@
       <c r="B27" s="93"/>
       <c r="C27" s="94"/>
       <c r="D27" s="95" t="str">
-        <v>query3 rejects</v>
+        <v>query3 error:7</v>
       </c>
       <c r="E27" s="100"/>
       <c r="F27" s="97"/>
@@ -9605,7 +9605,7 @@
       <c r="B28" s="93"/>
       <c r="C28" s="94"/>
       <c r="D28" s="95" t="str">
-        <v>query4 rejects</v>
+        <v>query4 error:7</v>
       </c>
       <c r="E28" s="100"/>
       <c r="F28" s="97"/>
@@ -9634,7 +9634,7 @@
       <c r="B29" s="93"/>
       <c r="C29" s="94"/>
       <c r="D29" s="95" t="str">
-        <v>valid OTP</v>
+        <v>valid OTP:1</v>
       </c>
       <c r="E29" s="100"/>
       <c r="F29" s="97"/>
@@ -9714,53 +9714,53 @@
       <c r="B32" s="112"/>
       <c r="C32" s="113"/>
       <c r="D32" s="114" t="str">
-        <v>HTTP code (C5)</v>
+        <v>HTTP as input</v>
       </c>
       <c r="E32" s="115"/>
-      <c r="F32" s="97" t="n">
-        <v>3</v>
-      </c>
-      <c r="G32" s="97" t="n">
-        <v>3</v>
-      </c>
-      <c r="H32" s="97" t="n">
-        <v>6</v>
-      </c>
-      <c r="I32" s="97" t="n">
-        <v>1</v>
-      </c>
-      <c r="J32" s="97" t="n">
-        <v>3</v>
-      </c>
-      <c r="K32" s="97" t="n">
-        <v>3</v>
-      </c>
-      <c r="L32" s="97" t="n">
-        <v>3</v>
-      </c>
-      <c r="M32" s="97" t="n">
-        <v>1</v>
-      </c>
-      <c r="N32" s="97" t="n">
-        <v>1</v>
-      </c>
-      <c r="O32" s="97" t="n">
-        <v>1</v>
-      </c>
-      <c r="P32" s="97" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q32" s="97" t="n">
-        <v>7</v>
-      </c>
-      <c r="R32" s="97" t="n">
-        <v>7</v>
-      </c>
-      <c r="S32" s="97" t="n">
-        <v>7</v>
-      </c>
-      <c r="T32" s="247" t="n">
-        <v>1</v>
+      <c r="F32" s="97" t="str">
+        <v>O</v>
+      </c>
+      <c r="G32" s="97" t="str">
+        <v>O</v>
+      </c>
+      <c r="H32" s="97" t="str">
+        <v>O</v>
+      </c>
+      <c r="I32" s="97" t="str">
+        <v>O</v>
+      </c>
+      <c r="J32" s="97" t="str">
+        <v>O</v>
+      </c>
+      <c r="K32" s="97" t="str">
+        <v>O</v>
+      </c>
+      <c r="L32" s="97" t="str">
+        <v>O</v>
+      </c>
+      <c r="M32" s="97" t="str">
+        <v>O</v>
+      </c>
+      <c r="N32" s="97" t="str">
+        <v>O</v>
+      </c>
+      <c r="O32" s="97" t="str">
+        <v>O</v>
+      </c>
+      <c r="P32" s="97" t="str">
+        <v>O</v>
+      </c>
+      <c r="Q32" s="97" t="str">
+        <v>O</v>
+      </c>
+      <c r="R32" s="97" t="str">
+        <v>O</v>
+      </c>
+      <c r="S32" s="97" t="str">
+        <v>O</v>
+      </c>
+      <c r="T32" s="247" t="str">
+        <v>O</v>
       </c>
       <c r="U32"/>
       <c r="V32"/>
@@ -10617,7 +10617,7 @@
     <row r="14" spans="1:23" ht="13.5" customHeight="1">
       <c r="A14" s="279"/>
       <c r="B14" s="130" t="str">
-        <v>Input / state</v>
+        <v>Input/state : HTTP</v>
       </c>
       <c r="C14" s="131"/>
       <c r="D14" s="132"/>
@@ -10643,7 +10643,7 @@
       <c r="B15" s="130"/>
       <c r="C15" s="131"/>
       <c r="D15" s="132" t="str">
-        <v>email=""</v>
+        <v>email="":3</v>
       </c>
       <c r="E15" s="137"/>
       <c r="F15" s="134" t="str">
@@ -10672,7 +10672,7 @@
       <c r="B16" s="130"/>
       <c r="C16" s="131"/>
       <c r="D16" s="132" t="str">
-        <v>password=""</v>
+        <v>pwd="":3</v>
       </c>
       <c r="E16" s="137"/>
       <c r="F16" s="134"/>
@@ -10701,7 +10701,7 @@
       <c r="B17" s="130"/>
       <c r="C17" s="131"/>
       <c r="D17" s="132" t="str">
-        <v>user not found</v>
+        <v>user not found:3</v>
       </c>
       <c r="E17" s="137"/>
       <c r="F17" s="134"/>
@@ -10730,7 +10730,7 @@
       <c r="B18" s="130"/>
       <c r="C18" s="131"/>
       <c r="D18" s="132" t="str">
-        <v>status=LOCKED</v>
+        <v>status=LOCKED:5</v>
       </c>
       <c r="E18" s="137"/>
       <c r="F18" s="134"/>
@@ -10759,7 +10759,7 @@
       <c r="B19" s="130"/>
       <c r="C19" s="131"/>
       <c r="D19" s="404" t="str">
-        <v>SUSPENDED</v>
+        <v>SUSPEND:5</v>
       </c>
       <c r="E19" s="404"/>
       <c r="F19" s="134"/>
@@ -10788,7 +10788,7 @@
       <c r="B20" s="130"/>
       <c r="C20" s="131"/>
       <c r="D20" s="132" t="str">
-        <v>wrong password</v>
+        <v>wrong pwd:3</v>
       </c>
       <c r="E20" s="137"/>
       <c r="F20" s="134"/>
@@ -10817,7 +10817,7 @@
       <c r="B21" s="130"/>
       <c r="C21" s="131"/>
       <c r="D21" s="132" t="str">
-        <v>verified=false</v>
+        <v>verified=false:4</v>
       </c>
       <c r="E21" s="137"/>
       <c r="F21" s="134"/>
@@ -10846,7 +10846,7 @@
       <c r="B22" s="130"/>
       <c r="C22" s="131"/>
       <c r="D22" s="132" t="str">
-        <v>FREELANCER hash</v>
+        <v>FREE hash:1</v>
       </c>
       <c r="E22" s="137"/>
       <c r="F22" s="134"/>
@@ -10875,7 +10875,7 @@
       <c r="B23" s="130"/>
       <c r="C23" s="131"/>
       <c r="D23" s="132" t="str">
-        <v>ADMIN plain pwd</v>
+        <v>ADMIN plain:1</v>
       </c>
       <c r="E23" s="137"/>
       <c r="F23" s="134"/>
@@ -10904,7 +10904,7 @@
       <c r="B24" s="130"/>
       <c r="C24" s="131"/>
       <c r="D24" s="132" t="str">
-        <v>ADMIN bcrypt</v>
+        <v>ADMIN bcrypt:1</v>
       </c>
       <c r="E24" s="137"/>
       <c r="F24" s="134"/>
@@ -10933,7 +10933,7 @@
       <c r="B25" s="130"/>
       <c r="C25" s="131"/>
       <c r="D25" s="132" t="str">
-        <v>query1 rejects</v>
+        <v>query1 error:7</v>
       </c>
       <c r="E25" s="137"/>
       <c r="F25" s="134"/>
@@ -10962,7 +10962,7 @@
       <c r="B26" s="130"/>
       <c r="C26" s="131"/>
       <c r="D26" s="132" t="str">
-        <v>query2 rejects</v>
+        <v>query2 error:7</v>
       </c>
       <c r="E26" s="137"/>
       <c r="F26" s="134"/>
@@ -10991,7 +10991,7 @@
       <c r="B27" s="130"/>
       <c r="C27" s="131"/>
       <c r="D27" s="132" t="str">
-        <v>query3 rejects</v>
+        <v>query3 error:7</v>
       </c>
       <c r="E27" s="137"/>
       <c r="F27" s="134"/>
@@ -11020,7 +11020,7 @@
       <c r="B28" s="130"/>
       <c r="C28" s="131"/>
       <c r="D28" s="132" t="str">
-        <v>JWT sign throws</v>
+        <v>JWT sign throws:7</v>
       </c>
       <c r="E28" s="137"/>
       <c r="F28" s="134"/>
@@ -11049,7 +11049,7 @@
       <c r="B29" s="130"/>
       <c r="C29" s="131"/>
       <c r="D29" s="132" t="str">
-        <v>OTP save rejects</v>
+        <v>OTP save error:7</v>
       </c>
       <c r="E29" s="137"/>
       <c r="F29" s="134"/>
@@ -11129,53 +11129,53 @@
       <c r="B32" s="149"/>
       <c r="C32" s="150"/>
       <c r="D32" s="151" t="str">
-        <v>HTTP code (C5)</v>
+        <v>HTTP as input</v>
       </c>
       <c r="E32" s="152"/>
-      <c r="F32" s="134" t="n">
-        <v>3</v>
-      </c>
-      <c r="G32" s="134" t="n">
-        <v>3</v>
-      </c>
-      <c r="H32" s="134" t="n">
-        <v>3</v>
-      </c>
-      <c r="I32" s="134" t="n">
-        <v>5</v>
-      </c>
-      <c r="J32" s="134" t="n">
-        <v>5</v>
-      </c>
-      <c r="K32" s="134" t="n">
-        <v>3</v>
-      </c>
-      <c r="L32" s="134" t="n">
-        <v>4</v>
-      </c>
-      <c r="M32" s="134" t="n">
-        <v>1</v>
-      </c>
-      <c r="N32" s="134" t="n">
-        <v>1</v>
-      </c>
-      <c r="O32" s="134" t="n">
-        <v>1</v>
-      </c>
-      <c r="P32" s="134" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q32" s="134" t="n">
-        <v>7</v>
-      </c>
-      <c r="R32" s="134" t="n">
-        <v>7</v>
-      </c>
-      <c r="S32" s="134" t="n">
-        <v>7</v>
-      </c>
-      <c r="T32" s="278" t="n">
-        <v>7</v>
+      <c r="F32" s="134" t="str">
+        <v>O</v>
+      </c>
+      <c r="G32" s="134" t="str">
+        <v>O</v>
+      </c>
+      <c r="H32" s="134" t="str">
+        <v>O</v>
+      </c>
+      <c r="I32" s="134" t="str">
+        <v>O</v>
+      </c>
+      <c r="J32" s="134" t="str">
+        <v>O</v>
+      </c>
+      <c r="K32" s="134" t="str">
+        <v>O</v>
+      </c>
+      <c r="L32" s="134" t="str">
+        <v>O</v>
+      </c>
+      <c r="M32" s="134" t="str">
+        <v>O</v>
+      </c>
+      <c r="N32" s="134" t="str">
+        <v>O</v>
+      </c>
+      <c r="O32" s="134" t="str">
+        <v>O</v>
+      </c>
+      <c r="P32" s="134" t="str">
+        <v>O</v>
+      </c>
+      <c r="Q32" s="134" t="str">
+        <v>O</v>
+      </c>
+      <c r="R32" s="134" t="str">
+        <v>O</v>
+      </c>
+      <c r="S32" s="134" t="str">
+        <v>O</v>
+      </c>
+      <c r="T32" s="278" t="str">
+        <v>O</v>
       </c>
       <c r="U32"/>
       <c r="V32"/>

</xml_diff>